<commit_message>
style: update ResultStatusLegend theme for light mode support and update sample MCQ template
</commit_message>
<xml_diff>
--- a/frontend/public/templates/sample_mcq_upload.xlsx
+++ b/frontend/public/templates/sample_mcq_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -491,45 +491,25 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Option 1 Image</t>
+          <t>Option 2</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Option 2</t>
+          <t>Option 3</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Option 2 Image</t>
+          <t>Option 4</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Option 3</t>
+          <t>Correct Option</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Option 3 Image</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Option 4</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Option 4 Image</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Correct Option</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Explanation</t>
         </is>
@@ -561,43 +541,23 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>data_chart_1.png</t>
+          <t>7</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>data_chart_2.png</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_3.png</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_4.png</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Simple multiplication of 1 and 5.</t>
         </is>
@@ -629,43 +589,23 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>data_chart_1.png</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>data_chart_2.png</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_3.png</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_4.png</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Simple multiplication of 2 and 5.</t>
         </is>
@@ -697,43 +637,23 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>data_chart_1.png</t>
+          <t>17</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>data_chart_2.png</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_3.png</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_4.png</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Simple multiplication of 3 and 5.</t>
         </is>
@@ -765,43 +685,23 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>data_chart_1.png</t>
+          <t>22</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>15</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>data_chart_2.png</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_3.png</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_4.png</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Simple multiplication of 4 and 5.</t>
         </is>
@@ -833,43 +733,23 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>data_chart_1.png</t>
+          <t>27</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>20</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>data_chart_2.png</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_3.png</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>data_chart_4.png</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Simple multiplication of 5 and 5.</t>
         </is>

</xml_diff>